<commit_message>
baseline: re-ratify drift gate — hormuz re-tilt RESTORE BOTH (owner ruling 2026-07-14 EVE) + same-evening price vintage
Drift decomposition: the ruled reweight (TRMD HOLD->BUY +9.1pp, STNG
TRIM->HOLD +7.3pp — both eyeballed as RULED-FV flips in their logs;
HAFN/CCEC/FLNG move without flips; ASC boundary eyeballed, NO flip at
+4.0%) + the 18:30 price vintage (EV-only, dNAV +0.0 all rows). The
proposal's what-if reproduced to the cent on all five bands. 2343 now
live-priced (static-fallback cleared on tonight's cron). Outputs regen
from clean HEAD (stamp 893002d); five families re-stamped current.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.39</v>
+        <v>0.3905</v>
       </c>
     </row>
     <row r="5">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>18773.65598239033</v>
+        <v>18872.23278046139</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.183411954691614</v>
+        <v>1.189625819556397</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
close(week): Week-close 7/13-7/18 — doc audit applied (5-agent fan-out), ratified spot re-proxy WIRED (dry-bulk band-mech flips CMDB/GNK/SBLK), price vintage annotated x16, PLAN rewritten for the 7/20 Week, baltic override, CHANGELOG entry
crude-tanker-fv. Full detail in the CHANGELOG 2026-07-18 entry. Gate at commit: suite
589+15xf green (hygiene clean-stamp regen follows), drift 0 UNEXPLAINED / 17 explained,
reconcile 25x SANITY-OK. Includes the daily-churn set (prices/manifest/ffa-queue).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3905</v>
+        <v>0.3955</v>
       </c>
     </row>
     <row r="5">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>18872.23278046139</v>
+        <v>19858.00076117199</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.189625819556397</v>
+        <v>1.251764468204235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ingest(containers): container_mb_refresh W28+W29 PROMOTED at owner go — Ctr-Feeder 12M 23,750→24,250 (1,700 cell 30k→31k, the ONE mover) on all three surfaces (12M/spot-mirror/strip re-synthesis); value curves comment-restamped W29 flat (NAV FROZEN book-wide, verified); as_of default→7/17 with dry-bulk 7/13 holds per convention; §11.8.5 feeder cycle 1.14x→1.16x; trigger re-armed 8/21; gate 0 unexplained / 11 explained (7/21-close price catch-up annotated; GNK recross eyeballed)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3955</v>
+        <v>0.3941</v>
       </c>
     </row>
     <row r="5">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>18543.26972405819</v>
+        <v>18266.98808919579</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.167761448809284</v>
+        <v>1.150362627187888</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ingest(dry-bulk): 24-Jul FFA promotion at owner go — full human eyeball of all flagged OCR rows (7/21-24; 100% of misreads were inside flagged rows), Cape/Pana/Supra fronts promoted on all three surfaces, Supra Cal27-derived strip legs HELD at 7/13 (source viewport crops Smax Cal27 — vintage_notes bracket), Handy-Bulk x0.90 regenerated, as_of default -> 7/24; FFA-only deltas verified at constant prices: 6 dry-bulk names, scenario FV -0.4..-0.7%, no band flips, NAV frozen
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3820010382057028</v>
+        <v>0.3826379651187989</v>
       </c>
     </row>
     <row r="6">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.36515925204608</v>
+        <v>0.3667515693288203</v>
       </c>
     </row>
     <row r="9">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>14902.5</v>
+        <v>15097.5</v>
       </c>
     </row>
     <row r="11">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.224061327440027</v>
+        <v>1.23981025730694</v>
       </c>
     </row>
     <row r="12">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>18266.98808919579</v>
+        <v>18360.32526336631</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.150362627187888</v>
+        <v>1.141328379021843</v>
       </c>
     </row>
   </sheetData>
@@ -826,19 +826,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>16920</v>
+        <v>17190</v>
       </c>
       <c r="C2" t="n">
-        <v>16920</v>
+        <v>17190</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02138628550712342</v>
+        <v>0.02193201326066176</v>
       </c>
       <c r="E2" t="n">
-        <v>0.02138628550712342</v>
+        <v>0.02193201326066176</v>
       </c>
       <c r="F2" t="n">
-        <v>0.02083553304379164</v>
+        <v>0.02136720688860096</v>
       </c>
     </row>
     <row r="3">
@@ -848,19 +848,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>16090</v>
+        <v>16600</v>
       </c>
       <c r="C3" t="n">
-        <v>16090</v>
+        <v>16600</v>
       </c>
       <c r="D3" t="n">
-        <v>0.01967642995772066</v>
+        <v>0.02073986207041808</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01967642995772066</v>
+        <v>0.02073986207041808</v>
       </c>
       <c r="F3" t="n">
-        <v>0.01867604082223457</v>
+        <v>0.0196854059149413</v>
       </c>
     </row>
     <row r="4">
@@ -876,13 +876,13 @@
         <v>13570</v>
       </c>
       <c r="D4" t="n">
-        <v>0.01441557327835332</v>
+        <v>0.01442542860053563</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01441557327835332</v>
+        <v>0.01442542860053563</v>
       </c>
       <c r="F4" t="n">
-        <v>0.01333029265251052</v>
+        <v>0.01333940601389672</v>
       </c>
     </row>
     <row r="5">
@@ -898,13 +898,13 @@
         <v>13030</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01328983838977299</v>
+        <v>0.01329969371195529</v>
       </c>
       <c r="E5" t="n">
-        <v>0.01328983838977299</v>
+        <v>0.01329969371195529</v>
       </c>
       <c r="F5" t="n">
-        <v>0.01197282737817387</v>
+        <v>0.01198170604680657</v>
       </c>
     </row>
     <row r="6">
@@ -920,13 +920,13 @@
         <v>12490</v>
       </c>
       <c r="D6" t="n">
-        <v>0.01216410350119266</v>
+        <v>0.01217395882337496</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01216410350119266</v>
+        <v>0.01217395882337496</v>
       </c>
       <c r="F6" t="n">
-        <v>0.01067643802277785</v>
+        <v>0.01068508804260574</v>
       </c>
     </row>
     <row r="7">
@@ -942,13 +942,13 @@
         <v>11950</v>
       </c>
       <c r="D7" t="n">
-        <v>0.01103836861261233</v>
+        <v>0.01104822393479463</v>
       </c>
       <c r="E7" t="n">
-        <v>0.01103836861261233</v>
+        <v>0.01104822393479463</v>
       </c>
       <c r="F7" t="n">
-        <v>0.009438879124976946</v>
+        <v>0.009447306384301316</v>
       </c>
     </row>
     <row r="8">
@@ -964,13 +964,13 @@
         <v>11680</v>
       </c>
       <c r="D8" t="n">
-        <v>0.01047550116832217</v>
+        <v>0.01048535649050447</v>
       </c>
       <c r="E8" t="n">
-        <v>0.01047550116832217</v>
+        <v>0.01048535649050447</v>
       </c>
       <c r="F8" t="n">
-        <v>0.008726891907142756</v>
+        <v>0.008735102142625817</v>
       </c>
     </row>
     <row r="9">
@@ -986,13 +986,13 @@
         <v>11410</v>
       </c>
       <c r="D9" t="n">
-        <v>0.009912633724032</v>
+        <v>0.009922489046214305</v>
       </c>
       <c r="E9" t="n">
-        <v>0.009912633724032</v>
+        <v>0.009922489046214305</v>
       </c>
       <c r="F9" t="n">
-        <v>0.008045315902955928</v>
+        <v>0.008053314703525934</v>
       </c>
     </row>
     <row r="10">
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.1017022188545641</v>
+        <v>0.1032945361373044</v>
       </c>
     </row>
     <row r="11">
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.36515925204608</v>
+        <v>0.3667515693288203</v>
       </c>
     </row>
     <row r="13">
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>14902.5</v>
+        <v>15097.5</v>
       </c>
     </row>
   </sheetData>
@@ -1053,7 +1053,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
@@ -1099,19 +1099,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2818479122382087</v>
+        <v>0.282293761077376</v>
       </c>
       <c r="C2" t="n">
-        <v>0.319854692303912</v>
+        <v>0.3203005411430793</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3578614723696152</v>
+        <v>0.3583073212087824</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3958682524353184</v>
+        <v>0.3963141012744857</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4338750325010216</v>
+        <v>0.4343208813401889</v>
       </c>
     </row>
     <row r="3">
@@ -1121,19 +1121,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.2939176951562525</v>
+        <v>0.2944590830323843</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3319244752219558</v>
+        <v>0.3324658630980875</v>
       </c>
       <c r="D3" t="n">
-        <v>0.369931255287659</v>
+        <v>0.3704726431637907</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4079380353533623</v>
+        <v>0.4084794232294939</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4459448154190654</v>
+        <v>0.4464862032951971</v>
       </c>
     </row>
     <row r="4">
@@ -1143,19 +1143,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3059874780742964</v>
+        <v>0.3066244049873925</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3439942581399997</v>
+        <v>0.3446311850530958</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3820010382057028</v>
+        <v>0.3826379651187989</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4200078182714061</v>
+        <v>0.4206447451845022</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4580145983371092</v>
+        <v>0.4586515252502054</v>
       </c>
     </row>
     <row r="5">
@@ -1165,19 +1165,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3180572609923402</v>
+        <v>0.3187897269424007</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3560640410580435</v>
+        <v>0.3567965070081041</v>
       </c>
       <c r="D5" t="n">
-        <v>0.3940708211237466</v>
+        <v>0.3948032870738072</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4320776011894499</v>
+        <v>0.4328100671395104</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4700843812551531</v>
+        <v>0.4708168472052136</v>
       </c>
     </row>
     <row r="6">
@@ -1187,19 +1187,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3301270439103841</v>
+        <v>0.330955048897409</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3681338239760873</v>
+        <v>0.3689618289631122</v>
       </c>
       <c r="D6" t="n">
-        <v>0.4061406040417905</v>
+        <v>0.4069686090288155</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4441473841074938</v>
+        <v>0.4449753890945187</v>
       </c>
       <c r="F6" t="n">
-        <v>0.4821541641731969</v>
+        <v>0.4829821691602219</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
baseline: re-ratify drift gate — week-close batch absorb 2026-07-26: 7/21+7/24-close price vintages EV-only (dNAV 0.0 every row; SB -1.5% = 7/18 marks-snapshot residual) + container W28/W29 promote (sub-display) + 7/24 FFA promote (sub-2pp); five flips eyeballed INDIVIDUALLY: SBLK BUY->HOLD price-at-FV (coherent w/ governance take-profit), GNK tender-pinned recross (outcome PR pending Mon 7/28), ASC pre-warned oscillation, GSL recross, 2343 rally crossing - all band-mech
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3941</v>
+        <v>0.4208</v>
       </c>
     </row>
     <row r="5">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>18360.32526336631</v>
+        <v>23656.33369689721</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.141328379021843</v>
+        <v>1.470542847394479</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
promote(marks-trail): 7/28 batch at owner go — 12 transactions/14 prints into Cape+Pana+Supra-Ultra per the §G-amended triage; prompt_premium flag SHIPPED (QUALITY_UPLIFT + template, in_fit:false on the 4 young prints — fitted Supra age-5 $30.9M vs $38M NB-parity cap, G1 satisfied); AEGIR 15.9->16.2 newest-wins; CMB JORDAENS cmbt_log disposal note; NAV +0.4..+2.6% on 6 dry-bulk names, NO flips (G6 freeze untriggered); 2343_log reordered newest-first (auto-prepend anchor quirk, flagged for its own fix)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3826379651187989</v>
+        <v>0.3879299690447122</v>
       </c>
     </row>
     <row r="6">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.3932288956454514</v>
+        <v>0.3994381887161819</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.3667515693288203</v>
+        <v>0.3706676395375078</v>
       </c>
     </row>
     <row r="9">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.23981025730694</v>
+        <v>1.241312575901231</v>
       </c>
     </row>
     <row r="12">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>23656.33369689721</v>
+        <v>22622.25497756105</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.470542847394479</v>
+        <v>1.405291751548208</v>
       </c>
     </row>
   </sheetData>
@@ -611,7 +611,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1086.500847409869</v>
+        <v>1118.36920768018</v>
       </c>
     </row>
     <row r="4">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>22.8310833087486</v>
+        <v>23.03526043021122</v>
       </c>
     </row>
     <row r="5">
@@ -722,7 +722,7 @@
         <v/>
       </c>
       <c r="B11" t="n">
-        <v>2031.124689308784</v>
+        <v>2063.197226700558</v>
       </c>
     </row>
     <row r="12">
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.3932288956454514</v>
+        <v>0.3994381887161819</v>
       </c>
     </row>
     <row r="14">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.3932288956454514</v>
+        <v>0.3994381887161819</v>
       </c>
     </row>
     <row r="15">
@@ -1012,10 +1012,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.333185811639983</v>
+        <v>0.3381383422864973</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2634570331915159</v>
+        <v>0.2673731034002034</v>
       </c>
     </row>
     <row r="12">
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.3667515693288203</v>
+        <v>0.3706676395375078</v>
       </c>
     </row>
     <row r="13">
@@ -1053,7 +1053,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
@@ -1099,19 +1099,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.282293761077376</v>
+        <v>0.2865273642181067</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3203005411430793</v>
+        <v>0.3250633446764013</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3583073212087824</v>
+        <v>0.3635993251346957</v>
       </c>
       <c r="E2" t="n">
-        <v>0.3963141012744857</v>
+        <v>0.4021353055929905</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4343208813401889</v>
+        <v>0.440671286051285</v>
       </c>
     </row>
     <row r="3">
@@ -1121,19 +1121,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.2944590830323843</v>
+        <v>0.298692686173115</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3324658630980875</v>
+        <v>0.3372286666314095</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3704726431637907</v>
+        <v>0.375764647089704</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4084794232294939</v>
+        <v>0.4143006275479987</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4464862032951971</v>
+        <v>0.4528366080062932</v>
       </c>
     </row>
     <row r="4">
@@ -1143,19 +1143,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3066244049873925</v>
+        <v>0.3108580081281232</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3446311850530958</v>
+        <v>0.3493939885864178</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3826379651187989</v>
+        <v>0.3879299690447122</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4206447451845022</v>
+        <v>0.426465949503007</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4586515252502054</v>
+        <v>0.4650019299613015</v>
       </c>
     </row>
     <row r="5">
@@ -1165,19 +1165,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3187897269424007</v>
+        <v>0.3230233300831314</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3567965070081041</v>
+        <v>0.361559310541426</v>
       </c>
       <c r="D5" t="n">
-        <v>0.3948032870738072</v>
+        <v>0.4000952909997205</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4328100671395104</v>
+        <v>0.4386312714580152</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4708168472052136</v>
+        <v>0.4771672519163097</v>
       </c>
     </row>
     <row r="6">
@@ -1187,19 +1187,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.330955048897409</v>
+        <v>0.3351886520381396</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3689618289631122</v>
+        <v>0.3737246324964343</v>
       </c>
       <c r="D6" t="n">
-        <v>0.4069686090288155</v>
+        <v>0.4122606129547287</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4449753890945187</v>
+        <v>0.4507965934130235</v>
       </c>
       <c r="F6" t="n">
-        <v>0.4829821691602219</v>
+        <v>0.489332573871318</v>
       </c>
     </row>
   </sheetData>
@@ -1237,7 +1237,7 @@
         <v>0.8</v>
       </c>
       <c r="B2" t="n">
-        <v>0.38</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="3">
@@ -1245,7 +1245,7 @@
         <v>0.95</v>
       </c>
       <c r="B3" t="n">
-        <v>0.38</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="4">
@@ -1253,7 +1253,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="n">
-        <v>0.38</v>
+        <v>0.39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
reweight(crude): B' regen at live 7/31 prices + gate annotations (9 rows, TNK flip eyeballed, CAPT no-flip rider recorded) + baseline ratify (RATIFY_LOG row); crude Set A' registered in the §9.10 family; stale-price artifact regen discarded
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4208</v>
+        <v>0.4183</v>
       </c>
     </row>
     <row r="5">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>22622.25497756105</v>
+        <v>22126.03178719314</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.405291751548208</v>
+        <v>1.374466426794215</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(outputs): clean-stamp regen after the 2343 refresh (at HEAD^)
2343 NAV 0.41 / TRIM/SHORT on the committed Q2 surface (11 names at Q2
vintage, 14 lagging, disclosed); dry-bulk family current. Gate 0/0. Suite
green.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -460,7 +460,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-Q1</t>
+          <t>2026-Q2</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3879299690447122</v>
+        <v>0.3995951798169115</v>
       </c>
     </row>
     <row r="6">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.3994381887161819</v>
+        <v>0.4105505086107764</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.3706676395375078</v>
+        <v>0.3831621866261141</v>
       </c>
     </row>
     <row r="9">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.241312575901231</v>
+        <v>1.23966087990904</v>
       </c>
     </row>
     <row r="12">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>35266.02186813492</v>
+        <v>32650.26077212765</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2.190721026279928</v>
+        <v>2.030002436646879</v>
       </c>
     </row>
   </sheetData>
@@ -611,7 +611,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -633,7 +633,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1140.218758590167</v>
+        <v>1166.50958042911</v>
       </c>
     </row>
     <row r="3">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1118.36920768018</v>
+        <v>1127.209092284535</v>
       </c>
     </row>
     <row r="4">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>23.03526043021122</v>
+        <v>22.30043990870066</v>
       </c>
     </row>
     <row r="5">
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>270.559</v>
+        <v>206.53</v>
       </c>
     </row>
     <row r="6">
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>26.362</v>
+        <v>85.83799999999999</v>
       </c>
     </row>
     <row r="7">
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-136.521</v>
+        <v>-49.309</v>
       </c>
     </row>
     <row r="8">
@@ -693,7 +693,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-93.90000000000001</v>
+        <v>-93.95699999999999</v>
       </c>
     </row>
     <row r="9">
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-284.926</v>
+        <v>-344.526</v>
       </c>
     </row>
     <row r="10">
@@ -722,7 +722,7 @@
         <v/>
       </c>
       <c r="B11" t="n">
-        <v>2063.197226700558</v>
+        <v>2120.595112622345</v>
       </c>
     </row>
     <row r="12">
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.3994381887161819</v>
+        <v>0.4105505086107764</v>
       </c>
     </row>
     <row r="14">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.3994381887161819</v>
+        <v>0.4105505086107764</v>
       </c>
     </row>
     <row r="15">
@@ -832,13 +832,13 @@
         <v>17190</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02193201326066176</v>
+        <v>0.02235617513412067</v>
       </c>
       <c r="E2" t="n">
-        <v>0.02193201326066176</v>
+        <v>0.02235617513412067</v>
       </c>
       <c r="F2" t="n">
-        <v>0.02136720688860096</v>
+        <v>0.02178044549085501</v>
       </c>
     </row>
     <row r="3">
@@ -854,13 +854,13 @@
         <v>16600</v>
       </c>
       <c r="D3" t="n">
-        <v>0.02073986207041808</v>
+        <v>0.02114379910878983</v>
       </c>
       <c r="E3" t="n">
-        <v>0.02073986207041808</v>
+        <v>0.02114379910878983</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0196854059149413</v>
+        <v>0.02006880598469243</v>
       </c>
     </row>
     <row r="4">
@@ -876,13 +876,13 @@
         <v>13570</v>
       </c>
       <c r="D4" t="n">
-        <v>0.01442542860053563</v>
+        <v>0.01472549911295127</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01442542860053563</v>
+        <v>0.01472549911295127</v>
       </c>
       <c r="F4" t="n">
-        <v>0.01333940601389672</v>
+        <v>0.01361688563053436</v>
       </c>
     </row>
     <row r="5">
@@ -898,13 +898,13 @@
         <v>13030</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01329969371195529</v>
+        <v>0.01358125335835896</v>
       </c>
       <c r="E5" t="n">
-        <v>0.01329969371195529</v>
+        <v>0.01358125335835896</v>
       </c>
       <c r="F5" t="n">
-        <v>0.01198170604680657</v>
+        <v>0.01223536338590898</v>
       </c>
     </row>
     <row r="6">
@@ -920,13 +920,13 @@
         <v>12490</v>
       </c>
       <c r="D6" t="n">
-        <v>0.01217395882337496</v>
+        <v>0.01243700760376665</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01217395882337496</v>
+        <v>0.01243700760376665</v>
       </c>
       <c r="F6" t="n">
-        <v>0.01068508804260574</v>
+        <v>0.01091596605186831</v>
       </c>
     </row>
     <row r="7">
@@ -942,13 +942,13 @@
         <v>11950</v>
       </c>
       <c r="D7" t="n">
-        <v>0.01104822393479463</v>
+        <v>0.01129276184917434</v>
       </c>
       <c r="E7" t="n">
-        <v>0.01104822393479463</v>
+        <v>0.01129276184917434</v>
       </c>
       <c r="F7" t="n">
-        <v>0.009447306384301316</v>
+        <v>0.009656410093038382</v>
       </c>
     </row>
     <row r="8">
@@ -964,13 +964,13 @@
         <v>11680</v>
       </c>
       <c r="D8" t="n">
-        <v>0.01048535649050447</v>
+        <v>0.01072063897187819</v>
       </c>
       <c r="E8" t="n">
-        <v>0.01048535649050447</v>
+        <v>0.01072063897187819</v>
       </c>
       <c r="F8" t="n">
-        <v>0.008735102142625817</v>
+        <v>0.008931110405104171</v>
       </c>
     </row>
     <row r="9">
@@ -986,13 +986,13 @@
         <v>11410</v>
       </c>
       <c r="D9" t="n">
-        <v>0.009922489046214305</v>
+        <v>0.01014851609458204</v>
       </c>
       <c r="E9" t="n">
-        <v>0.009922489046214305</v>
+        <v>0.01014851609458204</v>
       </c>
       <c r="F9" t="n">
-        <v>0.008053314703525934</v>
+        <v>0.008236763326501124</v>
       </c>
     </row>
     <row r="10">
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.1032945361373044</v>
+        <v>0.1054417503685027</v>
       </c>
     </row>
     <row r="11">
@@ -1012,10 +1012,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.3381383422864973</v>
+        <v>0.351224288236167</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2673731034002034</v>
+        <v>0.2777204362576113</v>
       </c>
     </row>
     <row r="12">
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.3706676395375078</v>
+        <v>0.3831621866261141</v>
       </c>
     </row>
     <row r="13">
@@ -1099,19 +1099,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2865273642181067</v>
+        <v>0.2964485404300728</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3250633446764013</v>
+        <v>0.3356571097361787</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3635993251346957</v>
+        <v>0.3748656790422846</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4021353055929905</v>
+        <v>0.4140742483483905</v>
       </c>
       <c r="F2" t="n">
-        <v>0.440671286051285</v>
+        <v>0.4532828176544965</v>
       </c>
     </row>
     <row r="3">
@@ -1121,19 +1121,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.298692686173115</v>
+        <v>0.3088132908173863</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3372286666314095</v>
+        <v>0.3480218601234921</v>
       </c>
       <c r="D3" t="n">
-        <v>0.375764647089704</v>
+        <v>0.3872304294295981</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4143006275479987</v>
+        <v>0.4264389987357039</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4528366080062932</v>
+        <v>0.46564756804181</v>
       </c>
     </row>
     <row r="4">
@@ -1143,19 +1143,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3108580081281232</v>
+        <v>0.3211780412046997</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3493939885864178</v>
+        <v>0.3603866105108056</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3879299690447122</v>
+        <v>0.3995951798169115</v>
       </c>
       <c r="E4" t="n">
-        <v>0.426465949503007</v>
+        <v>0.4388037491230173</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4650019299613015</v>
+        <v>0.4780123184291234</v>
       </c>
     </row>
     <row r="5">
@@ -1165,19 +1165,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3230233300831314</v>
+        <v>0.3335427915920131</v>
       </c>
       <c r="C5" t="n">
-        <v>0.361559310541426</v>
+        <v>0.372751360898119</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4000952909997205</v>
+        <v>0.4119599302042249</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4386312714580152</v>
+        <v>0.4511684995103307</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4771672519163097</v>
+        <v>0.4903770688164368</v>
       </c>
     </row>
     <row r="6">
@@ -1187,19 +1187,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3351886520381396</v>
+        <v>0.3459075419793265</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3737246324964343</v>
+        <v>0.3851161112854324</v>
       </c>
       <c r="D6" t="n">
-        <v>0.4122606129547287</v>
+        <v>0.4243246805915383</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4507965934130235</v>
+        <v>0.4635332498976442</v>
       </c>
       <c r="F6" t="n">
-        <v>0.489332573871318</v>
+        <v>0.5027418192037503</v>
       </c>
     </row>
   </sheetData>
@@ -1237,7 +1237,7 @@
         <v>0.8</v>
       </c>
       <c r="B2" t="n">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="3">
@@ -1245,7 +1245,7 @@
         <v>0.95</v>
       </c>
       <c r="B3" t="n">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="4">
@@ -1253,7 +1253,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="n">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clean-stamp regen after the marks-trail promotion (outputs + log entries)
book_scorecard source_commit clean at adf7a6e; drift gate 0 UNEXPLAINED,
delta report 0 material. Broker-sweep header reflects the re-pinned k band.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -425,7 +425,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3995951798169115</v>
+        <v>0.3998750435000599</v>
       </c>
     </row>
     <row r="6">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.4105505086107764</v>
+        <v>0.4108768485591928</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.3831621866261141</v>
+        <v>0.3833723359113606</v>
       </c>
     </row>
     <row r="9">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.23966087990904</v>
+        <v>1.239746540277111</v>
       </c>
     </row>
     <row r="12">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>32650.26077212765</v>
+        <v>32598.77994758524</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2.030002436646879</v>
+        <v>2.026607337582418</v>
       </c>
     </row>
   </sheetData>
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1127.209092284535</v>
+        <v>1128.743838888087</v>
       </c>
     </row>
     <row r="4">
@@ -653,7 +653,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>22.30043990870066</v>
+        <v>22.45132000673705</v>
       </c>
     </row>
     <row r="5">
@@ -722,7 +722,7 @@
         <v/>
       </c>
       <c r="B11" t="n">
-        <v>2120.595112622345</v>
+        <v>2122.280739323935</v>
       </c>
     </row>
     <row r="12">
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.4105505086107764</v>
+        <v>0.4108768485591928</v>
       </c>
     </row>
     <row r="14">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.4105505086107764</v>
+        <v>0.4108768485591928</v>
       </c>
     </row>
     <row r="15">
@@ -1012,10 +1012,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.351224288236167</v>
+        <v>0.3514900574180417</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2777204362576113</v>
+        <v>0.2779305855428579</v>
       </c>
     </row>
     <row r="12">
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.3831621866261141</v>
+        <v>0.3833723359113606</v>
       </c>
     </row>
     <row r="13">
@@ -1099,19 +1099,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2964485404300728</v>
+        <v>0.2966724313765917</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3356571097361787</v>
+        <v>0.3359089870510124</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3748656790422846</v>
+        <v>0.3751455427254331</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4140742483483905</v>
+        <v>0.414382098399854</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4532828176544965</v>
+        <v>0.4536186540742747</v>
       </c>
     </row>
     <row r="3">
@@ -1121,19 +1121,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3088132908173863</v>
+        <v>0.3090371817639052</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3480218601234921</v>
+        <v>0.3482737374383258</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3872304294295981</v>
+        <v>0.3875102931127465</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4264389987357039</v>
+        <v>0.4267468487871673</v>
       </c>
       <c r="F3" t="n">
-        <v>0.46564756804181</v>
+        <v>0.4659834044615881</v>
       </c>
     </row>
     <row r="4">
@@ -1143,19 +1143,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3211780412046997</v>
+        <v>0.3214019321512186</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3603866105108056</v>
+        <v>0.3606384878256392</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3995951798169115</v>
+        <v>0.3998750435000599</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4388037491230173</v>
+        <v>0.4391115991744808</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4780123184291234</v>
+        <v>0.4783481548489015</v>
       </c>
     </row>
     <row r="5">
@@ -1165,19 +1165,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3335427915920131</v>
+        <v>0.333766682538532</v>
       </c>
       <c r="C5" t="n">
-        <v>0.372751360898119</v>
+        <v>0.3730032382129527</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4119599302042249</v>
+        <v>0.4122397938873733</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4511684995103307</v>
+        <v>0.4514763495617942</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4903770688164368</v>
+        <v>0.4907129052362149</v>
       </c>
     </row>
     <row r="6">
@@ -1187,19 +1187,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3459075419793265</v>
+        <v>0.3461314329258455</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3851161112854324</v>
+        <v>0.3853679886002661</v>
       </c>
       <c r="D6" t="n">
-        <v>0.4243246805915383</v>
+        <v>0.4246045442746867</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4635332498976442</v>
+        <v>0.4638410999491076</v>
       </c>
       <c r="F6" t="n">
-        <v>0.5027418192037503</v>
+        <v>0.5030776556235284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clean-stamp regen: FFA + container promotions' outputs, fresh family sidecars
Family diagnostics re-run (crude robustness / product / LNG) after the
promotion round — weight_sign_stable coverage restored; hygiene + vintage
guards green; drift gate 0 UNEXPLAINED; full suite 636 passed / 15 xfailed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -425,7 +425,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="39" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3998750435000599</v>
+        <v>0.406064827343163</v>
       </c>
     </row>
     <row r="6">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.3833723359113606</v>
+        <v>0.4012528061271332</v>
       </c>
     </row>
     <row r="9">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>15097.5</v>
+        <v>15280</v>
       </c>
     </row>
     <row r="11">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.239746540277111</v>
+        <v>1.166449296152441</v>
       </c>
     </row>
     <row r="12">
@@ -552,7 +552,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>elevated</t>
+          <t>mid-cycle</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="14">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="15">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>32598.77994758524</v>
+        <v>28574.03649196291</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2.026607337582418</v>
+        <v>1.755065863312244</v>
       </c>
     </row>
   </sheetData>
@@ -826,19 +826,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17190</v>
+        <v>17280</v>
       </c>
       <c r="C2" t="n">
-        <v>17190</v>
+        <v>17280</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02235617513412067</v>
+        <v>0.02261087093869289</v>
       </c>
       <c r="E2" t="n">
-        <v>0.02235617513412067</v>
+        <v>0.02261087093869289</v>
       </c>
       <c r="F2" t="n">
-        <v>0.02178044549085501</v>
+        <v>0.02202858221616488</v>
       </c>
     </row>
     <row r="3">
@@ -848,19 +848,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>16600</v>
+        <v>17240</v>
       </c>
       <c r="C3" t="n">
-        <v>16600</v>
+        <v>17240</v>
       </c>
       <c r="D3" t="n">
-        <v>0.02114379910878983</v>
+        <v>0.02250299372510086</v>
       </c>
       <c r="E3" t="n">
-        <v>0.02114379910878983</v>
+        <v>0.02250299372510086</v>
       </c>
       <c r="F3" t="n">
-        <v>0.02006880598469243</v>
+        <v>0.02135889642254779</v>
       </c>
     </row>
     <row r="4">
@@ -876,13 +876,13 @@
         <v>13570</v>
       </c>
       <c r="D4" t="n">
-        <v>0.01472549911295127</v>
+        <v>0.01464322859734248</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01472549911295127</v>
+        <v>0.01464322859734248</v>
       </c>
       <c r="F4" t="n">
-        <v>0.01361688563053436</v>
+        <v>0.01354080887461478</v>
       </c>
     </row>
     <row r="5">
@@ -898,13 +898,13 @@
         <v>13030</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01358125335835896</v>
+        <v>0.0136078198790243</v>
       </c>
       <c r="E5" t="n">
-        <v>0.01358125335835896</v>
+        <v>0.0136078198790243</v>
       </c>
       <c r="F5" t="n">
-        <v>0.01223536338590898</v>
+        <v>0.01225929718831018</v>
       </c>
     </row>
     <row r="6">
@@ -920,13 +920,13 @@
         <v>12490</v>
       </c>
       <c r="D6" t="n">
-        <v>0.01243700760376665</v>
+        <v>0.01248114230745262</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01243700760376665</v>
+        <v>0.01248114230745262</v>
       </c>
       <c r="F6" t="n">
-        <v>0.01091596605186831</v>
+        <v>0.01095470309718453</v>
       </c>
     </row>
     <row r="7">
@@ -942,13 +942,13 @@
         <v>11950</v>
       </c>
       <c r="D7" t="n">
-        <v>0.01129276184917434</v>
+        <v>0.01135403624361214</v>
       </c>
       <c r="E7" t="n">
-        <v>0.01129276184917434</v>
+        <v>0.01135403624361214</v>
       </c>
       <c r="F7" t="n">
-        <v>0.009656410093038382</v>
+        <v>0.0097088056618812</v>
       </c>
     </row>
     <row r="8">
@@ -964,13 +964,13 @@
         <v>11680</v>
       </c>
       <c r="D8" t="n">
-        <v>0.01072063897187819</v>
+        <v>0.01078191336631599</v>
       </c>
       <c r="E8" t="n">
-        <v>0.01072063897187819</v>
+        <v>0.01078191336631599</v>
       </c>
       <c r="F8" t="n">
-        <v>0.008931110405104171</v>
+        <v>0.008982156651803217</v>
       </c>
     </row>
     <row r="9">
@@ -986,13 +986,13 @@
         <v>11410</v>
       </c>
       <c r="D9" t="n">
-        <v>0.01014851609458204</v>
+        <v>0.01020979048901983</v>
       </c>
       <c r="E9" t="n">
-        <v>0.01014851609458204</v>
+        <v>0.01020979048901983</v>
       </c>
       <c r="F9" t="n">
-        <v>0.008236763326501124</v>
+        <v>0.008286494999610285</v>
       </c>
     </row>
     <row r="10">
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.1054417503685027</v>
+        <v>0.1071197451121169</v>
       </c>
     </row>
     <row r="11">
@@ -1012,10 +1012,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.3514900574180417</v>
+        <v>0.3719808178102446</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2779305855428579</v>
+        <v>0.2941330610150163</v>
       </c>
     </row>
     <row r="12">
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.3833723359113606</v>
+        <v>0.4012528061271332</v>
       </c>
     </row>
     <row r="13">
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>15097.5</v>
+        <v>15280</v>
       </c>
     </row>
   </sheetData>
@@ -1099,19 +1099,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2966724313765917</v>
+        <v>0.2976251773597201</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3359089870510124</v>
+        <v>0.3362632147615287</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3751455427254331</v>
+        <v>0.3749012521633373</v>
       </c>
       <c r="E2" t="n">
-        <v>0.414382098399854</v>
+        <v>0.4135392895651461</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4536186540742747</v>
+        <v>0.4521773269669548</v>
       </c>
     </row>
     <row r="3">
@@ -1121,19 +1121,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3090371817639052</v>
+        <v>0.3132069649496329</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3482737374383258</v>
+        <v>0.3518450023514414</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3875102931127465</v>
+        <v>0.3904830397532502</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4267468487871673</v>
+        <v>0.4291210771550589</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4659834044615881</v>
+        <v>0.4677591145568676</v>
       </c>
     </row>
     <row r="4">
@@ -1143,19 +1143,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3214019321512186</v>
+        <v>0.3287887525395458</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3606384878256392</v>
+        <v>0.3674267899413543</v>
       </c>
       <c r="D4" t="n">
-        <v>0.3998750435000599</v>
+        <v>0.406064827343163</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4391115991744808</v>
+        <v>0.4447028647449718</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4783481548489015</v>
+        <v>0.4833409021467804</v>
       </c>
     </row>
     <row r="5">
@@ -1165,19 +1165,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.333766682538532</v>
+        <v>0.3443705401294586</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3730032382129527</v>
+        <v>0.3830085775312672</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4122397938873733</v>
+        <v>0.4216466149330758</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4514763495617942</v>
+        <v>0.4602846523348846</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4907129052362149</v>
+        <v>0.4989226897366933</v>
       </c>
     </row>
     <row r="6">
@@ -1187,19 +1187,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3461314329258455</v>
+        <v>0.3599523277193715</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3853679886002661</v>
+        <v>0.39859036512118</v>
       </c>
       <c r="D6" t="n">
-        <v>0.4246045442746867</v>
+        <v>0.4372284025229887</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4638410999491076</v>
+        <v>0.4758664399247974</v>
       </c>
       <c r="F6" t="n">
-        <v>0.5030776556235284</v>
+        <v>0.5145044773266061</v>
       </c>
     </row>
   </sheetData>
@@ -1245,7 +1245,7 @@
         <v>0.95</v>
       </c>
       <c r="B3" t="n">
-        <v>0.4</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="4">
@@ -1253,7 +1253,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="n">
-        <v>0.4</v>
+        <v>0.41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clean-stamp regen: WF Artemis retro-flag outputs (SBLK ratified-HOLD state)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.406064827343163</v>
+        <v>0.4028439403229644</v>
       </c>
     </row>
     <row r="6">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.4108768485591928</v>
+        <v>0.4069618932405875</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.4012528061271332</v>
+        <v>0.3987259874053414</v>
       </c>
     </row>
     <row r="9">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.166449296152441</v>
+        <v>1.166145425997569</v>
       </c>
     </row>
     <row r="12">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>28574.03649196291</v>
+        <v>29067.90300532554</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.755065863312244</v>
+        <v>1.786072129457378</v>
       </c>
     </row>
   </sheetData>
@@ -611,7 +611,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1128.743838888087</v>
+        <v>1108.522124529817</v>
       </c>
     </row>
     <row r="4">
@@ -722,7 +722,7 @@
         <v/>
       </c>
       <c r="B11" t="n">
-        <v>2122.280739323935</v>
+        <v>2102.059024965665</v>
       </c>
     </row>
     <row r="12">
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.4108768485591928</v>
+        <v>0.4069618932405875</v>
       </c>
     </row>
     <row r="14">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.4108768485591928</v>
+        <v>0.4069618932405875</v>
       </c>
     </row>
     <row r="15">
@@ -1012,10 +1012,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.3719808178102446</v>
+        <v>0.3687852297612617</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2941330610150163</v>
+        <v>0.2916062422932245</v>
       </c>
     </row>
     <row r="12">
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.4012528061271332</v>
+        <v>0.3987259874053414</v>
       </c>
     </row>
     <row r="13">
@@ -1099,19 +1099,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2976251773597201</v>
+        <v>0.2950484677435611</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3362632147615287</v>
+        <v>0.3333644164433497</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3749012521633373</v>
+        <v>0.3716803651431387</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4135392895651461</v>
+        <v>0.4099963138429273</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4521773269669548</v>
+        <v>0.4483122625427162</v>
       </c>
     </row>
     <row r="3">
@@ -1121,19 +1121,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3132069649496329</v>
+        <v>0.3106302553334739</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3518450023514414</v>
+        <v>0.3489462040332625</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3904830397532502</v>
+        <v>0.3872621527330515</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4291210771550589</v>
+        <v>0.4255781014328401</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4677591145568676</v>
+        <v>0.463894050132629</v>
       </c>
     </row>
     <row r="4">
@@ -1143,19 +1143,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3287887525395458</v>
+        <v>0.3262120429233868</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3674267899413543</v>
+        <v>0.3645279916231754</v>
       </c>
       <c r="D4" t="n">
-        <v>0.406064827343163</v>
+        <v>0.4028439403229644</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4447028647449718</v>
+        <v>0.441159889022753</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4833409021467804</v>
+        <v>0.4794758377225419</v>
       </c>
     </row>
     <row r="5">
@@ -1165,19 +1165,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3443705401294586</v>
+        <v>0.3417938305132996</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3830085775312672</v>
+        <v>0.3801097792130882</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4216466149330758</v>
+        <v>0.4184257279128772</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4602846523348846</v>
+        <v>0.4567416766126658</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4989226897366933</v>
+        <v>0.4950576253124547</v>
       </c>
     </row>
     <row r="6">
@@ -1187,19 +1187,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3599523277193715</v>
+        <v>0.3573756181032124</v>
       </c>
       <c r="C6" t="n">
-        <v>0.39859036512118</v>
+        <v>0.3956915668030011</v>
       </c>
       <c r="D6" t="n">
-        <v>0.4372284025229887</v>
+        <v>0.4340075155027901</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4758664399247974</v>
+        <v>0.4723234642025787</v>
       </c>
       <c r="F6" t="n">
-        <v>0.5145044773266061</v>
+        <v>0.5106394129023676</v>
       </c>
     </row>
   </sheetData>
@@ -1245,7 +1245,7 @@
         <v>0.95</v>
       </c>
       <c r="B3" t="n">
-        <v>0.41</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="4">
@@ -1253,7 +1253,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="n">
-        <v>0.41</v>
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
outputs: BRUT H1 pair regen (pre-clean-stamp)
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4845</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="5">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>29067.90300532554</v>
+        <v>14262.49103180476</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.786072129457378</v>
+        <v>0.8763562243851994</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Absorb the 8/25 clean-HEAD regen (verified: stamp dcf02a3, hygiene 2/2, family sidecars re-run) + gap-week automation deltas (8/26-8/28 log prepends, baltic tape, Pareto manifest)
The uncommitted regen sat through 8/26-8/29 and the price cron's dirty-tree
guard correctly refused to write — the book is 3 sessions stale as a result;
manual 8/28-close fetch follows as its own commit.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.4951</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="5">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>30728.61588277866</v>
+        <v>14262.49103180476</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.888114336798807</v>
+        <v>0.8763562243851994</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rebase-promote regen: 8/28 vintage live book-wide, flips eyeballed (2343 guard-release T/S, CAPT/CMDB price-led, TNK k=pnav-re-pin, SB edge deflated to honest ~+25%), 8 gate rows annotated — 11 EV%-only rows ride the owner ratify
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -471,7 +471,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.39</v>
+        <v>0.5326</v>
       </c>
     </row>
     <row r="5">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>14262.49103180476</v>
+        <v>36603.77936433452</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.8763562243851994</v>
+        <v>2.24911271182745</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FFA-promote regen: predicted-impact addendum (cycle-reweight channel missed — recorded), SBLK+CMDB 12M-leg flips FROZEN-FOR-OWNER-REVIEW per G6; dry EV -3pp = the elevated-cycle fade, mechanism verified in attribution
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.4028439403229644</v>
+        <v>0.4055781183804164</v>
       </c>
     </row>
     <row r="6">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.3987259874053414</v>
+        <v>0.4035024560901597</v>
       </c>
     </row>
     <row r="9">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>15280</v>
+        <v>15921</v>
       </c>
     </row>
     <row r="11">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.166145425997569</v>
+        <v>1.201121947038584</v>
       </c>
     </row>
     <row r="12">
@@ -552,7 +552,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>mid-cycle</t>
+          <t>elevated</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="14">
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="15">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>36603.77936433452</v>
+        <v>40554.42983500702</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2.24911271182745</v>
+        <v>2.389068815999797</v>
       </c>
     </row>
   </sheetData>
@@ -826,19 +826,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17280</v>
+        <v>17505</v>
       </c>
       <c r="C2" t="n">
-        <v>17280</v>
+        <v>17505</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02261087093869289</v>
+        <v>0.02312357050815244</v>
       </c>
       <c r="E2" t="n">
-        <v>0.02261087093869289</v>
+        <v>0.02312357050815244</v>
       </c>
       <c r="F2" t="n">
-        <v>0.02202858221616488</v>
+        <v>0.02252807843851982</v>
       </c>
     </row>
     <row r="3">
@@ -848,19 +848,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>17240</v>
+        <v>18248</v>
       </c>
       <c r="C3" t="n">
-        <v>17240</v>
+        <v>18248</v>
       </c>
       <c r="D3" t="n">
-        <v>0.02250299372510086</v>
+        <v>0.02468780724492764</v>
       </c>
       <c r="E3" t="n">
-        <v>0.02250299372510086</v>
+        <v>0.02468780724492764</v>
       </c>
       <c r="F3" t="n">
-        <v>0.02135889642254779</v>
+        <v>0.02343262964411955</v>
       </c>
     </row>
     <row r="4">
@@ -870,19 +870,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13570</v>
+        <v>13635</v>
       </c>
       <c r="C4" t="n">
-        <v>13570</v>
+        <v>13635</v>
       </c>
       <c r="D4" t="n">
-        <v>0.01464322859734248</v>
+        <v>0.01483022262344497</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01464322859734248</v>
+        <v>0.01483022262344497</v>
       </c>
       <c r="F4" t="n">
-        <v>0.01354080887461478</v>
+        <v>0.01371372500109033</v>
       </c>
     </row>
     <row r="5">
@@ -892,19 +892,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>13030</v>
+        <v>14296</v>
       </c>
       <c r="C5" t="n">
-        <v>13030</v>
+        <v>14296</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0136078198790243</v>
+        <v>0.01629347230231038</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0136078198790243</v>
+        <v>0.01629347230231038</v>
       </c>
       <c r="F5" t="n">
-        <v>0.01225929718831018</v>
+        <v>0.01467880387595529</v>
       </c>
     </row>
     <row r="6">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12490</v>
+        <v>14295</v>
       </c>
       <c r="C6" t="n">
-        <v>12490</v>
+        <v>14295</v>
       </c>
       <c r="D6" t="n">
-        <v>0.01248114230745262</v>
+        <v>0.01629148409818316</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01248114230745262</v>
+        <v>0.01629148409818316</v>
       </c>
       <c r="F6" t="n">
-        <v>0.01095470309718453</v>
+        <v>0.01429904145885223</v>
       </c>
     </row>
     <row r="7">
@@ -936,19 +936,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>11950</v>
+        <v>14295</v>
       </c>
       <c r="C7" t="n">
-        <v>11950</v>
+        <v>14295</v>
       </c>
       <c r="D7" t="n">
-        <v>0.01135403624361214</v>
+        <v>0.01629148409818316</v>
       </c>
       <c r="E7" t="n">
-        <v>0.01135403624361214</v>
+        <v>0.01629148409818316</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0097088056618812</v>
+        <v>0.01393080395897769</v>
       </c>
     </row>
     <row r="8">
@@ -958,19 +958,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>11680</v>
+        <v>14025</v>
       </c>
       <c r="C8" t="n">
-        <v>11680</v>
+        <v>14025</v>
       </c>
       <c r="D8" t="n">
-        <v>0.01078191336631599</v>
+        <v>0.01571936122088701</v>
       </c>
       <c r="E8" t="n">
-        <v>0.01078191336631599</v>
+        <v>0.01571936122088701</v>
       </c>
       <c r="F8" t="n">
-        <v>0.008982156651803217</v>
+        <v>0.01309542751413625</v>
       </c>
     </row>
     <row r="9">
@@ -980,19 +980,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11410</v>
+        <v>13755</v>
       </c>
       <c r="C9" t="n">
-        <v>11410</v>
+        <v>13755</v>
       </c>
       <c r="D9" t="n">
-        <v>0.01020979048901983</v>
+        <v>0.01514723834359085</v>
       </c>
       <c r="E9" t="n">
-        <v>0.01020979048901983</v>
+        <v>0.01514723834359085</v>
       </c>
       <c r="F9" t="n">
-        <v>0.008286494999610285</v>
+        <v>0.01229383844135285</v>
       </c>
     </row>
     <row r="10">
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.1071197451121169</v>
+        <v>0.127972348333004</v>
       </c>
     </row>
     <row r="11">
@@ -1012,10 +1012,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.3687852297612617</v>
+        <v>0.3484542487715079</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2916062422932245</v>
+        <v>0.2755301077571557</v>
       </c>
     </row>
     <row r="12">
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.3987259874053414</v>
+        <v>0.4035024560901597</v>
       </c>
     </row>
     <row r="13">
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>15280</v>
+        <v>15921</v>
       </c>
     </row>
   </sheetData>
@@ -1099,19 +1099,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2950484677435611</v>
+        <v>0.3003336673622967</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3333644164433497</v>
+        <v>0.3392393066061729</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3716803651431387</v>
+        <v>0.3781449458500493</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4099963138429273</v>
+        <v>0.4170505850939255</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4483122625427162</v>
+        <v>0.4559562243378018</v>
       </c>
     </row>
     <row r="3">
@@ -1121,19 +1121,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3106302553334739</v>
+        <v>0.3140502536274802</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3489462040332625</v>
+        <v>0.3529558928713563</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3872621527330515</v>
+        <v>0.3918615321152329</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4255781014328401</v>
+        <v>0.430767171359109</v>
       </c>
       <c r="F3" t="n">
-        <v>0.463894050132629</v>
+        <v>0.4696728106029853</v>
       </c>
     </row>
     <row r="4">
@@ -1143,19 +1143,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3262120429233868</v>
+        <v>0.3277668398926638</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3645279916231754</v>
+        <v>0.3666724791365398</v>
       </c>
       <c r="D4" t="n">
-        <v>0.4028439403229644</v>
+        <v>0.4055781183804164</v>
       </c>
       <c r="E4" t="n">
-        <v>0.441159889022753</v>
+        <v>0.4444837576242925</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4794758377225419</v>
+        <v>0.4833893968681688</v>
       </c>
     </row>
     <row r="5">
@@ -1165,19 +1165,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3417938305132996</v>
+        <v>0.3414834261578472</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3801097792130882</v>
+        <v>0.3803890654017233</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4184257279128772</v>
+        <v>0.4192947046455999</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4567416766126658</v>
+        <v>0.4582003438894759</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4950576253124547</v>
+        <v>0.4971059831333523</v>
       </c>
     </row>
     <row r="6">
@@ -1187,19 +1187,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3573756181032124</v>
+        <v>0.3552000124230308</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3956915668030011</v>
+        <v>0.3941056516669069</v>
       </c>
       <c r="D6" t="n">
-        <v>0.4340075155027901</v>
+        <v>0.4330112909107834</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4723234642025787</v>
+        <v>0.4719169301546595</v>
       </c>
       <c r="F6" t="n">
-        <v>0.5106394129023676</v>
+        <v>0.5108225693985358</v>
       </c>
     </row>
   </sheetData>
@@ -1245,7 +1245,7 @@
         <v>0.95</v>
       </c>
       <c r="B3" t="n">
-        <v>0.4</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="4">
@@ -1253,7 +1253,7 @@
         <v>1</v>
       </c>
       <c r="B4" t="n">
-        <v>0.4</v>
+        <v>0.41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Regen at the FFA-promote completion (Handy-Bulk rounding + as_of coherence): delta 0 material / 0 flips, gate 25 rows 0 UNEXPLAINED, strobe GNK -0.07% inside deadband unchanged — expected pipeline churn (25 decision-log model-state entries + outputs)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.4055781183804164</v>
+        <v>0.4055730139991362</v>
       </c>
     </row>
     <row r="6">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.4035024560901597</v>
+        <v>0.4034896951369593</v>
       </c>
     </row>
     <row r="9">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>15921</v>
+        <v>15922.5</v>
       </c>
     </row>
     <row r="11">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>40554.42983500702</v>
+        <v>40558.51331953585</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2.389068815999797</v>
+        <v>2.389202180803369</v>
       </c>
     </row>
   </sheetData>
@@ -826,19 +826,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17505</v>
+        <v>17500</v>
       </c>
       <c r="C2" t="n">
-        <v>17505</v>
+        <v>17500</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02312357050815244</v>
+        <v>0.02311808580711186</v>
       </c>
       <c r="E2" t="n">
-        <v>0.02312357050815244</v>
+        <v>0.02311808580711186</v>
       </c>
       <c r="F2" t="n">
-        <v>0.02252807843851982</v>
+        <v>0.02252273498279309</v>
       </c>
     </row>
     <row r="3">
@@ -848,19 +848,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18248</v>
+        <v>18250</v>
       </c>
       <c r="C3" t="n">
-        <v>18248</v>
+        <v>18250</v>
       </c>
       <c r="D3" t="n">
-        <v>0.02468780724492764</v>
+        <v>0.02469000112534388</v>
       </c>
       <c r="E3" t="n">
-        <v>0.02468780724492764</v>
+        <v>0.02469000112534388</v>
       </c>
       <c r="F3" t="n">
-        <v>0.02343262964411955</v>
+        <v>0.02343471198325834</v>
       </c>
     </row>
     <row r="4">
@@ -870,19 +870,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13635</v>
+        <v>13640</v>
       </c>
       <c r="C4" t="n">
-        <v>13635</v>
+        <v>13640</v>
       </c>
       <c r="D4" t="n">
-        <v>0.01483022262344497</v>
+        <v>0.01483570732448555</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01483022262344497</v>
+        <v>0.01483570732448555</v>
       </c>
       <c r="F4" t="n">
-        <v>0.01371372500109033</v>
+        <v>0.0137187967848183</v>
       </c>
     </row>
     <row r="5">
@@ -892,19 +892,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>14296</v>
+        <v>14300</v>
       </c>
       <c r="C5" t="n">
-        <v>14296</v>
+        <v>14300</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01629347230231038</v>
+        <v>0.01629786006314284</v>
       </c>
       <c r="E5" t="n">
-        <v>0.01629347230231038</v>
+        <v>0.01629786006314284</v>
       </c>
       <c r="F5" t="n">
-        <v>0.01467880387595529</v>
+        <v>0.0146827568136422</v>
       </c>
     </row>
     <row r="6">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14295</v>
+        <v>14290</v>
       </c>
       <c r="C6" t="n">
-        <v>14295</v>
+        <v>14290</v>
       </c>
       <c r="D6" t="n">
-        <v>0.01629148409818316</v>
+        <v>0.01628599939714257</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01629148409818316</v>
+        <v>0.01628599939714257</v>
       </c>
       <c r="F6" t="n">
-        <v>0.01429904145885223</v>
+        <v>0.01429422753477409</v>
       </c>
     </row>
     <row r="7">
@@ -936,19 +936,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>14295</v>
+        <v>14290</v>
       </c>
       <c r="C7" t="n">
-        <v>14295</v>
+        <v>14290</v>
       </c>
       <c r="D7" t="n">
-        <v>0.01629148409818316</v>
+        <v>0.01628599939714257</v>
       </c>
       <c r="E7" t="n">
-        <v>0.01629148409818316</v>
+        <v>0.01628599939714257</v>
       </c>
       <c r="F7" t="n">
-        <v>0.01393080395897769</v>
+        <v>0.01392611400596239</v>
       </c>
     </row>
     <row r="8">
@@ -958,19 +958,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>14025</v>
+        <v>14020</v>
       </c>
       <c r="C8" t="n">
-        <v>14025</v>
+        <v>14020</v>
       </c>
       <c r="D8" t="n">
-        <v>0.01571936122088701</v>
+        <v>0.01571387651984642</v>
       </c>
       <c r="E8" t="n">
-        <v>0.01571936122088701</v>
+        <v>0.01571387651984642</v>
       </c>
       <c r="F8" t="n">
-        <v>0.01309542751413625</v>
+        <v>0.01309085833960654</v>
       </c>
     </row>
     <row r="9">
@@ -980,19 +980,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>13755</v>
+        <v>13750</v>
       </c>
       <c r="C9" t="n">
-        <v>13755</v>
+        <v>13750</v>
       </c>
       <c r="D9" t="n">
-        <v>0.01514723834359085</v>
+        <v>0.01514175364255027</v>
       </c>
       <c r="E9" t="n">
-        <v>0.01514723834359085</v>
+        <v>0.01514175364255027</v>
       </c>
       <c r="F9" t="n">
-        <v>0.01229383844135285</v>
+        <v>0.01228938693494868</v>
       </c>
     </row>
     <row r="10">
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.127972348333004</v>
+        <v>0.1279595873798036</v>
       </c>
     </row>
     <row r="11">
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.4035024560901597</v>
+        <v>0.4034896951369593</v>
       </c>
     </row>
     <row r="13">
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>15921</v>
+        <v>15922.5</v>
       </c>
     </row>
   </sheetData>
@@ -1099,19 +1099,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.3003336673622967</v>
+        <v>0.3003300942954006</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3392393066061729</v>
+        <v>0.3392357335392767</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3781449458500493</v>
+        <v>0.3781413727831532</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4170505850939255</v>
+        <v>0.4170470120270294</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4559562243378018</v>
+        <v>0.4559526512709057</v>
       </c>
     </row>
     <row r="3">
@@ -1121,19 +1121,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3140502536274802</v>
+        <v>0.3140459149033921</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3529558928713563</v>
+        <v>0.3529515541472682</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3918615321152329</v>
+        <v>0.3918571933911447</v>
       </c>
       <c r="E3" t="n">
-        <v>0.430767171359109</v>
+        <v>0.4307628326350209</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4696728106029853</v>
+        <v>0.4696684718788972</v>
       </c>
     </row>
     <row r="4">
@@ -1143,19 +1143,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3277668398926638</v>
+        <v>0.3277617355113835</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3666724791365398</v>
+        <v>0.3666673747552597</v>
       </c>
       <c r="D4" t="n">
-        <v>0.4055781183804164</v>
+        <v>0.4055730139991362</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4444837576242925</v>
+        <v>0.4444786532430123</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4833893968681688</v>
+        <v>0.4833842924868886</v>
       </c>
     </row>
     <row r="5">
@@ -1165,19 +1165,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.3414834261578472</v>
+        <v>0.341477556119375</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3803890654017233</v>
+        <v>0.3803831953632512</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4192947046455999</v>
+        <v>0.4192888346071277</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4582003438894759</v>
+        <v>0.4581944738510038</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4971059831333523</v>
+        <v>0.4971001130948801</v>
       </c>
     </row>
     <row r="6">
@@ -1187,19 +1187,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3552000124230308</v>
+        <v>0.3551933767273665</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3941056516669069</v>
+        <v>0.3940990159712426</v>
       </c>
       <c r="D6" t="n">
-        <v>0.4330112909107834</v>
+        <v>0.4330046552151192</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4719169301546595</v>
+        <v>0.4719102944589952</v>
       </c>
       <c r="F6" t="n">
-        <v>0.5108225693985358</v>
+        <v>0.5108159337028716</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
S&P promotion round REGEN + close: ALL FROZEN BANDS HIT — dry five NAV +0.7/+1.0/+1.2/+1.2/+0.0% (SB/GNK/SBLK/CMDB/2343), EV fades -0.2..-1.1pp, NO flips (CMDB HOLD stands, the pre-eyeballed fade risk did not fire; SB BUY stands; the cycle channel predicted UP FRONT this time); non-dry EXACTLY 0.0 (forward invariance verified); GNK strobe crossed -0.07 -> +0.02% inside the deadband (surfaced, held on vintage per B2); all sub-gate-threshold — no new ratify row needed; five sidecars re-run; SBLK flip-margin re-pin -8.48 dated; CAPT test pins advanced to the Q2 pair (the morning refresh's leftover — first full suite since) + operating-scrubber ledger CAPT 5->8 BOTH surfaces (release-tied, agreement-guarded); mover logs annotated; gate 25 rows / 0 UNEXPLAINED / 1 explained (CAPT, rides R4 Phase 5); SUITE FULLY GREEN 701/13
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/2343_fv_report.xlsx
+++ b/outputs/2343_fv_report.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.4055730139991362</v>
+        <v>0.4112695494990081</v>
       </c>
     </row>
     <row r="6">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.4069618932405875</v>
+        <v>0.4109042754269337</v>
       </c>
     </row>
     <row r="8">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.4034896951369593</v>
+        <v>0.4118174606071197</v>
       </c>
     </row>
     <row r="9">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>15922.5</v>
+        <v>16420</v>
       </c>
     </row>
     <row r="11">
@@ -541,7 +541,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.201121947038584</v>
+        <v>1.228871369223343</v>
       </c>
     </row>
     <row r="12">
@@ -583,7 +583,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>40558.51331953585</v>
+        <v>40188.60260741775</v>
       </c>
     </row>
     <row r="16">
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2.389202180803369</v>
+        <v>2.293527065987367</v>
       </c>
     </row>
   </sheetData>
@@ -611,7 +611,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1108.522124529817</v>
+        <v>1128.885505456428</v>
       </c>
     </row>
     <row r="4">
@@ -722,7 +722,7 @@
         <v/>
       </c>
       <c r="B11" t="n">
-        <v>2102.059024965665</v>
+        <v>2122.422405892276</v>
       </c>
     </row>
     <row r="12">
@@ -742,7 +742,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.4069618932405875</v>
+        <v>0.4109042754269337</v>
       </c>
     </row>
     <row r="14">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.4069618932405875</v>
+        <v>0.4109042754269337</v>
       </c>
     </row>
     <row r="15">
@@ -826,19 +826,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17500</v>
+        <v>17890</v>
       </c>
       <c r="C2" t="n">
-        <v>17500</v>
+        <v>17890</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02311808580711186</v>
+        <v>0.02399215861638303</v>
       </c>
       <c r="E2" t="n">
-        <v>0.02311808580711186</v>
+        <v>0.02399215861638303</v>
       </c>
       <c r="F2" t="n">
-        <v>0.02252273498279309</v>
+        <v>0.02337429814434274</v>
       </c>
     </row>
     <row r="3">
@@ -848,19 +848,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18250</v>
+        <v>18840</v>
       </c>
       <c r="C3" t="n">
-        <v>18250</v>
+        <v>18840</v>
       </c>
       <c r="D3" t="n">
-        <v>0.02469000112534388</v>
+        <v>0.02596392578016455</v>
       </c>
       <c r="E3" t="n">
-        <v>0.02469000112534388</v>
+        <v>0.02596392578016455</v>
       </c>
       <c r="F3" t="n">
-        <v>0.02343471198325834</v>
+        <v>0.02464386775536763</v>
       </c>
     </row>
     <row r="4">
@@ -870,19 +870,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>13640</v>
+        <v>14400</v>
       </c>
       <c r="C4" t="n">
-        <v>13640</v>
+        <v>14400</v>
       </c>
       <c r="D4" t="n">
-        <v>0.01483570732448555</v>
+        <v>0.0164509517809382</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01483570732448555</v>
+        <v>0.0164509517809382</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0137187967848183</v>
+        <v>0.01521243709270613</v>
       </c>
     </row>
     <row r="5">
@@ -892,19 +892,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>14300</v>
+        <v>14550</v>
       </c>
       <c r="C5" t="n">
-        <v>14300</v>
+        <v>14550</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01629786006314284</v>
+        <v>0.01683690333728795</v>
       </c>
       <c r="E5" t="n">
-        <v>0.01629786006314284</v>
+        <v>0.01683690333728795</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0146827568136422</v>
+        <v>0.0151683813849441</v>
       </c>
     </row>
     <row r="6">
@@ -914,19 +914,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14290</v>
+        <v>14550</v>
       </c>
       <c r="C6" t="n">
-        <v>14290</v>
+        <v>14550</v>
       </c>
       <c r="D6" t="n">
-        <v>0.01628599939714257</v>
+        <v>0.0168368861975972</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01628599939714257</v>
+        <v>0.0168368861975972</v>
       </c>
       <c r="F6" t="n">
-        <v>0.01429422753477409</v>
+        <v>0.01477774107788424</v>
       </c>
     </row>
     <row r="7">
@@ -936,19 +936,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>14290</v>
+        <v>14550</v>
       </c>
       <c r="C7" t="n">
-        <v>14290</v>
+        <v>14550</v>
       </c>
       <c r="D7" t="n">
-        <v>0.01628599939714257</v>
+        <v>0.01683599493367811</v>
       </c>
       <c r="E7" t="n">
-        <v>0.01628599939714257</v>
+        <v>0.01683599493367811</v>
       </c>
       <c r="F7" t="n">
-        <v>0.01392611400596239</v>
+        <v>0.0143964137006749</v>
       </c>
     </row>
     <row r="8">
@@ -958,19 +958,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>14020</v>
+        <v>14280</v>
       </c>
       <c r="C8" t="n">
-        <v>14020</v>
+        <v>14280</v>
       </c>
       <c r="D8" t="n">
-        <v>0.01571387651984642</v>
+        <v>0.01626387205638196</v>
       </c>
       <c r="E8" t="n">
-        <v>0.01571387651984642</v>
+        <v>0.01626387205638196</v>
       </c>
       <c r="F8" t="n">
-        <v>0.01309085833960654</v>
+        <v>0.01354904659424308</v>
       </c>
     </row>
     <row r="9">
@@ -980,19 +980,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>13750</v>
+        <v>14010</v>
       </c>
       <c r="C9" t="n">
-        <v>13750</v>
+        <v>14010</v>
       </c>
       <c r="D9" t="n">
-        <v>0.01514175364255027</v>
+        <v>0.0156917491790858</v>
       </c>
       <c r="E9" t="n">
-        <v>0.01514175364255027</v>
+        <v>0.0156917491790858</v>
       </c>
       <c r="F9" t="n">
-        <v>0.01228938693494868</v>
+        <v>0.01273577565058502</v>
       </c>
     </row>
     <row r="10">
@@ -1002,7 +1002,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.1279595873798036</v>
+        <v>0.1338579614007478</v>
       </c>
     </row>
     <row r="11">
@@ -1012,10 +1012,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.3484542487715079</v>
+        <v>0.3515266236175797</v>
       </c>
       <c r="F11" t="n">
-        <v>0.2755301077571557</v>
+        <v>0.2779594992063718</v>
       </c>
     </row>
     <row r="12">
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.4034896951369593</v>
+        <v>0.4118174606071197</v>
       </c>
     </row>
     <row r="13">
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>15922.5</v>
+        <v>16420</v>
       </c>
     </row>
   </sheetData>
@@ -1099,19 +1099,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.3003300942954006</v>
+        <v>0.3046513877344604</v>
       </c>
       <c r="C2" t="n">
-        <v>0.3392357335392767</v>
+        <v>0.3438907455674861</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3781413727831532</v>
+        <v>0.3831301034005118</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4170470120270294</v>
+        <v>0.4223694612335374</v>
       </c>
       <c r="F2" t="n">
-        <v>0.4559526512709057</v>
+        <v>0.4616088190665631</v>
       </c>
     </row>
     <row r="3">
@@ -1121,19 +1121,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3140459149033921</v>
+        <v>0.3187211107837085</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3529515541472682</v>
+        <v>0.3579604686167343</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3918571933911447</v>
+        <v>0.3971998264497599</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4307628326350209</v>
+        <v>0.4364391842827855</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4696684718788972</v>
+        <v>0.4756785421158113</v>
       </c>
     </row>
     <row r="4">
@@ -1143,19 +1143,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.3277617355113835</v>
+        <v>0.3327908338329566</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3666673747552597</v>
+        <v>0.3720301916659824</v>
       </c>
       <c r="D4" t="n">
-        <v>0.4055730139991362</v>
+        <v>0.4112695494990081</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4444786532430123</v>
+        <v>0.4505089073320336</v>
       </c>
       <c r="F4" t="n">
-        <v>0.4833842924868886</v>
+        <v>0.4897482651650594</v>
       </c>
     </row>
     <row r="5">
@@ -1165,19 +1165,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.341477556119375</v>
+        <v>0.3468605568822047</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3803831953632512</v>
+        <v>0.3860999147152305</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4192888346071277</v>
+        <v>0.4253392725482562</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4581944738510038</v>
+        <v>0.4645786303812818</v>
       </c>
       <c r="F5" t="n">
-        <v>0.4971001130948801</v>
+        <v>0.5038179882143076</v>
       </c>
     </row>
     <row r="6">
@@ -1187,19 +1187,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.3551933767273665</v>
+        <v>0.3609302799314529</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3940990159712426</v>
+        <v>0.4001696377644787</v>
       </c>
       <c r="D6" t="n">
-        <v>0.4330046552151192</v>
+        <v>0.4394089955975043</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4719102944589952</v>
+        <v>0.4786483534305299</v>
       </c>
       <c r="F6" t="n">
-        <v>0.5108159337028716</v>
+        <v>0.5178877112635557</v>
       </c>
     </row>
   </sheetData>
@@ -1237,7 +1237,7 @@
         <v>0.8</v>
       </c>
       <c r="B2" t="n">
-        <v>0.4</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="3">

</xml_diff>